<commit_message>
test(estandarización): naming unificado, tags Playwright, stock fix, lista estrictos
- Formato unificado: describe 'MODULE-XX | Desc', test 'SC-XX: Desc @MODULE-XX.XX'
- Tags Playwright agregados: @busqueda, @facturacion+submodulo, @cierre-caja,
  @puntoventa+submodulos (Boleta/Factura/NV/NC/ND/Guias/Pedido/Cotización)
- Módulos estandarizados: BC, CC, FC, MS, NC, ND, PS, PV (incl. PV-18/19/20)
- llenarCantidadesStock: itera sobre todos .cmp-card-almacen (stock multi-almacén)
- LISTA_ITEMS_ESTRICTOS (447744) template en item-factory, helpers, setup
- Nuevos items: ESTRICTO_GRAVADO_1..10, EQUIVALENTE_SIN_CONTROL,
  VARIANTE_SIN_CONTROL + 'sin_control' type en controlStock
- EdicionItemPage: métodos para creación de selectores
- Import paths: relativos -> alias (@helpers, @app-types)
- CajaPage: esperarCargaOverlay en aperturarCajaResumido
- PuntoVentaSetupPage: timeout 30s en busqueda, remover emojis de logs
</commit_message>
<xml_diff>
--- a/src/data/FORMATO_EDICION_SERVICIOS_Masivos.xlsx
+++ b/src/data/FORMATO_EDICION_SERVICIOS_Masivos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\WebstormProjects\erpperu2-automation\src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31981456-2035-4DFF-B500-7B17EF014885}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3F7A9E9-70A9-43F7-855A-9598910F63D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2796" yWindow="0" windowWidth="10620" windowHeight="12384" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SERVICIOS" sheetId="1" r:id="rId1"/>
@@ -53,9 +53,6 @@
     <t>DESCRIPCION</t>
   </si>
   <si>
-    <t>PRECIO ESTANDAR</t>
-  </si>
-  <si>
     <t>Automatizados</t>
   </si>
   <si>
@@ -450,6 +447,9 @@
   </si>
   <si>
     <t>servicio automatizado X8</t>
+  </si>
+  <si>
+    <t>PRECIO ESTÁNDAR</t>
   </si>
 </sst>
 </file>
@@ -1255,31 +1255,31 @@
         <v>7</v>
       </c>
       <c r="I1" s="17" t="s">
-        <v>8</v>
+        <v>140</v>
       </c>
     </row>
     <row r="2" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B2" s="8"/>
       <c r="C2" s="9" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F2" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="G2" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="G2" s="9" t="s">
-        <v>10</v>
-      </c>
       <c r="H2" s="9" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="I2" s="18">
         <v>75</v>
@@ -1287,26 +1287,26 @@
     </row>
     <row r="3" spans="1:9" s="6" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="28" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B3" s="20"/>
       <c r="C3" s="21" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F3" s="10" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G3" s="21" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="H3" s="9" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="I3" s="22">
         <v>55.5</v>
@@ -1314,26 +1314,26 @@
     </row>
     <row r="4" spans="1:9" s="6" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="29" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B4" s="9"/>
       <c r="C4" s="9" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D4" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="I4" s="9">
         <v>48.9</v>
@@ -1341,26 +1341,26 @@
     </row>
     <row r="5" spans="1:9" s="6" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B5" s="19"/>
       <c r="C5" s="19" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D5" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F5" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="G5" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="G5" s="19" t="s">
-        <v>10</v>
-      </c>
       <c r="H5" s="9" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="I5" s="19">
         <v>120</v>
@@ -1368,26 +1368,26 @@
     </row>
     <row r="6" spans="1:9" s="6" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="28" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B6" s="19"/>
       <c r="C6" s="19" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F6" s="10" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G6" s="19" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="I6" s="19">
         <v>85</v>
@@ -1395,26 +1395,26 @@
     </row>
     <row r="7" spans="1:9" s="6" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="29" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B7" s="19"/>
       <c r="C7" s="19" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D7" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F7" s="10" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G7" s="19" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H7" s="9" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="I7" s="19">
         <v>60.5</v>
@@ -1422,26 +1422,26 @@
     </row>
     <row r="8" spans="1:9" s="6" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B8" s="19"/>
       <c r="C8" s="19" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D8" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F8" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="G8" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="G8" s="19" t="s">
-        <v>10</v>
-      </c>
       <c r="H8" s="9" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I8" s="19">
         <v>95</v>
@@ -1449,26 +1449,26 @@
     </row>
     <row r="9" spans="1:9" s="6" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="28" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B9" s="19"/>
       <c r="C9" s="19" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D9" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F9" s="10" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G9" s="19" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="H9" s="9" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="I9" s="19">
         <v>150</v>
@@ -2824,551 +2824,551 @@
     <row r="1" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B2" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="6" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B6" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B7" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B8" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="10" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="11" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B11" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="12" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B12" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="13" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="14" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="15" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B15" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="16" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B16" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="17" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="18" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="19" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="20" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B20" s="16" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="22" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="23" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B23" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="24" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B24" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="25" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B25" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="26" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="27" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B27" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="28" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B28" s="12" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="29" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B29" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="30" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B30" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="31" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B31" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="32" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B32" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="33" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B33" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="34" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B34" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="35" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B35" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="36" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B36" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="37" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B37" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="38" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B38" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="39" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B39" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="40" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B40" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="41" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B41" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="42" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B42" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="43" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B43" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="46" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="47" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B47" s="3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="48" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B48" s="12" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="49" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B49" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="50" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B50" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="51" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B51" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="52" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B52" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="54" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="55" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B55" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="56" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B56" s="12" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="57" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B57" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="58" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B58" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="59" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B59" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="60" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B60" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="61" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B61" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="62" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B62" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="63" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B63" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="64" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B64" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="65" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B65" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="66" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B66" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="67" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B67" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="68" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B68" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="69" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B69" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="70" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B70" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="71" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B71" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="72" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B72" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="73" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B73" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="74" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B74" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="75" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B75" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="76" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B76" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="77" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B77" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="78" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B78" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="79" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B79" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="80" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B80" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="81" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B81" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="82" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B82" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="83" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B83" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="84" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B84" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="85" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B85" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="86" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B86" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="87" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B87" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="88" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B88" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="89" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B89" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="90" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B90" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="91" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B91" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="92" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B92" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="93" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B93" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="94" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B94" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="95" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B95" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="96" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B96" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="97" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B97" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="98" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B98" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="99" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B99" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="100" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B100" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="101" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B101" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="102" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B102" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="103" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B103" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="104" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B104" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="105" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B105" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="106" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B106" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="107" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B107" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="108" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B108" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="109" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B109" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="110" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B110" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="111" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B111" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="112" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B112" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="113" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B113" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="114" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B114" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="115" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B115" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="116" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B116" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="117" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B117" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="119" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="120" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B120" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="121" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B121" s="12" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="122" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B122" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="123" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B123" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>